<commit_message>
updated after Malaysia NC
</commit_message>
<xml_diff>
--- a/pages/WR_progressions/Medals_Men_TP.xlsx
+++ b/pages/WR_progressions/Medals_Men_TP.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\WR_progressions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7B6A0FA-6F0E-4F41-AF28-9A111FFBCCD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6755DFDD-117F-49AA-9509-215DAE43DDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{60BF7A36-0D27-46A2-BCFD-CC0E6E4E1F78}"/>
+    <workbookView xWindow="25490" yWindow="10800" windowWidth="19420" windowHeight="10300" xr2:uid="{60BF7A36-0D27-46A2-BCFD-CC0E6E4E1F78}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="56">
   <si>
     <t>Year</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t>DateSerial</t>
+  </si>
+  <si>
+    <t>Santiago</t>
   </si>
 </sst>
 </file>
@@ -662,6 +665,9 @@
       <c r="B2" t="s">
         <v>40</v>
       </c>
+      <c r="C2" t="s">
+        <v>55</v>
+      </c>
       <c r="D2" s="1">
         <f>G2/86400</f>
         <v>2.5916087962962963E-3</v>

</xml_diff>